<commit_message>
update data Produksi TBS
</commit_message>
<xml_diff>
--- a/Produksi TBS.xlsx
+++ b/Produksi TBS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="22">
   <si>
     <t>PT</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>KEBUN LUAR</t>
+  </si>
+  <si>
+    <t>FFD</t>
   </si>
 </sst>
 </file>
@@ -2586,7 +2589,7 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>12</v>
@@ -2615,7 +2618,7 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>12</v>
@@ -2644,7 +2647,7 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>12</v>
@@ -2673,7 +2676,7 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>12</v>
@@ -2702,7 +2705,7 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>12</v>
@@ -2731,7 +2734,7 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>12</v>
@@ -2760,7 +2763,7 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>12</v>
@@ -2789,7 +2792,7 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>12</v>
@@ -2818,7 +2821,7 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>12</v>
@@ -2847,7 +2850,7 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>12</v>
@@ -2876,7 +2879,7 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>12</v>
@@ -2905,7 +2908,7 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>12</v>
@@ -2934,7 +2937,7 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>13</v>
@@ -2963,7 +2966,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>13</v>
@@ -2992,7 +2995,7 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>13</v>
@@ -3021,7 +3024,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>13</v>
@@ -3050,7 +3053,7 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>13</v>
@@ -3079,7 +3082,7 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>13</v>
@@ -3108,7 +3111,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>13</v>
@@ -3137,7 +3140,7 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>13</v>
@@ -3166,7 +3169,7 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>13</v>
@@ -3195,7 +3198,7 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>13</v>
@@ -3224,7 +3227,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>13</v>
@@ -3253,7 +3256,7 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>13</v>

</xml_diff>